<commit_message>
fix(tcs): revert TCS position window to T-2/T+4 per explicit request
Both FY27_Q2 and FY27_Q3 records (the dashboard duplicates the current
quarter's tracking across two quarter codes) had TCS on a walk-forward-
optimized T-6/T+1 window from an earlier explicit request. Reverted both
to the uniform T-2/T+4 window, recomputed entry/exit dates and prices
accordingly (entry 06-Oct-2026 @ Rs 2100.00, real price; exit 14-Oct-2026,
correctly still pending -- no fabricated price for a date that hasn't
happened yet).

Also: fixed stale "bias" (LONG/SHORT count) summary labels across all 18
quarters -- they hadn't been recalculated since BSE was added to the
universe, so every one was off by at least 1. No individual stock's
direction was changed, only the summary label.

fix_q3_position_window.py (the walk-forward optimizer that caused the
original override) has already been removed from the automated daily
pipeline so this won't recur on the next scheduled refresh.
</commit_message>
<xml_diff>
--- a/action_cop/output_excels/08_Company_Directory.xlsx
+++ b/action_cop/output_excels/08_Company_Directory.xlsx
@@ -458,7 +458,7 @@
       <c r="C2" t="inlineStr"/>
       <c r="D2" t="inlineStr">
         <is>
-          <t>2026-10-01 10:50:17</t>
+          <t>2026-10-08 16:16:03</t>
         </is>
       </c>
     </row>
@@ -476,7 +476,7 @@
       <c r="C3" t="inlineStr"/>
       <c r="D3" t="inlineStr">
         <is>
-          <t>2026-10-01 10:50:17</t>
+          <t>2026-10-08 16:16:03</t>
         </is>
       </c>
     </row>
@@ -494,7 +494,7 @@
       <c r="C4" t="inlineStr"/>
       <c r="D4" t="inlineStr">
         <is>
-          <t>2026-10-01 10:50:17</t>
+          <t>2026-10-08 16:16:03</t>
         </is>
       </c>
     </row>
@@ -512,7 +512,7 @@
       <c r="C5" t="inlineStr"/>
       <c r="D5" t="inlineStr">
         <is>
-          <t>2026-10-01 10:50:17</t>
+          <t>2026-10-08 16:16:03</t>
         </is>
       </c>
     </row>
@@ -530,7 +530,7 @@
       <c r="C6" t="inlineStr"/>
       <c r="D6" t="inlineStr">
         <is>
-          <t>2026-10-01 10:50:17</t>
+          <t>2026-10-08 16:16:03</t>
         </is>
       </c>
     </row>
@@ -552,7 +552,7 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>2026-10-01 10:50:17</t>
+          <t>2026-10-08 16:16:03</t>
         </is>
       </c>
     </row>
@@ -570,7 +570,7 @@
       <c r="C8" t="inlineStr"/>
       <c r="D8" t="inlineStr">
         <is>
-          <t>2026-10-01 10:50:17</t>
+          <t>2026-10-08 16:16:03</t>
         </is>
       </c>
     </row>
@@ -592,7 +592,7 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>2026-10-01 10:50:17</t>
+          <t>2026-10-08 16:16:03</t>
         </is>
       </c>
     </row>
@@ -610,7 +610,7 @@
       <c r="C10" t="inlineStr"/>
       <c r="D10" t="inlineStr">
         <is>
-          <t>2026-10-01 10:50:17</t>
+          <t>2026-10-08 16:16:03</t>
         </is>
       </c>
     </row>
@@ -628,7 +628,7 @@
       <c r="C11" t="inlineStr"/>
       <c r="D11" t="inlineStr">
         <is>
-          <t>2026-10-01 10:50:17</t>
+          <t>2026-10-08 16:16:03</t>
         </is>
       </c>
     </row>
@@ -646,7 +646,7 @@
       <c r="C12" t="inlineStr"/>
       <c r="D12" t="inlineStr">
         <is>
-          <t>2026-10-01 10:50:17</t>
+          <t>2026-10-08 16:16:03</t>
         </is>
       </c>
     </row>
@@ -664,7 +664,7 @@
       <c r="C13" t="inlineStr"/>
       <c r="D13" t="inlineStr">
         <is>
-          <t>2026-10-01 10:50:17</t>
+          <t>2026-10-08 16:16:03</t>
         </is>
       </c>
     </row>
@@ -682,7 +682,7 @@
       <c r="C14" t="inlineStr"/>
       <c r="D14" t="inlineStr">
         <is>
-          <t>2026-10-01 10:50:17</t>
+          <t>2026-10-08 16:16:03</t>
         </is>
       </c>
     </row>
@@ -700,7 +700,7 @@
       <c r="C15" t="inlineStr"/>
       <c r="D15" t="inlineStr">
         <is>
-          <t>2026-10-01 10:50:17</t>
+          <t>2026-10-08 16:16:03</t>
         </is>
       </c>
     </row>
@@ -722,7 +722,7 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>2026-10-01 10:50:17</t>
+          <t>2026-10-08 16:16:03</t>
         </is>
       </c>
     </row>
@@ -740,7 +740,7 @@
       <c r="C17" t="inlineStr"/>
       <c r="D17" t="inlineStr">
         <is>
-          <t>2026-10-01 10:50:17</t>
+          <t>2026-10-08 16:16:03</t>
         </is>
       </c>
     </row>
@@ -762,7 +762,7 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>2026-10-01 10:50:17</t>
+          <t>2026-10-08 16:16:03</t>
         </is>
       </c>
     </row>
@@ -780,7 +780,7 @@
       <c r="C19" t="inlineStr"/>
       <c r="D19" t="inlineStr">
         <is>
-          <t>2026-10-01 10:50:17</t>
+          <t>2026-10-08 16:16:03</t>
         </is>
       </c>
     </row>
@@ -798,7 +798,7 @@
       <c r="C20" t="inlineStr"/>
       <c r="D20" t="inlineStr">
         <is>
-          <t>2026-10-01 10:50:17</t>
+          <t>2026-10-08 16:16:03</t>
         </is>
       </c>
     </row>
@@ -816,7 +816,7 @@
       <c r="C21" t="inlineStr"/>
       <c r="D21" t="inlineStr">
         <is>
-          <t>2026-10-01 10:50:17</t>
+          <t>2026-10-08 16:16:03</t>
         </is>
       </c>
     </row>
@@ -838,7 +838,7 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>2026-10-01 10:50:17</t>
+          <t>2026-10-08 16:16:03</t>
         </is>
       </c>
     </row>
@@ -856,7 +856,7 @@
       <c r="C23" t="inlineStr"/>
       <c r="D23" t="inlineStr">
         <is>
-          <t>2026-10-01 10:50:17</t>
+          <t>2026-10-08 16:16:03</t>
         </is>
       </c>
     </row>
@@ -878,7 +878,7 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>2026-10-01 10:50:17</t>
+          <t>2026-10-08 16:16:03</t>
         </is>
       </c>
     </row>
@@ -900,7 +900,7 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>2026-10-01 10:50:17</t>
+          <t>2026-10-08 16:16:03</t>
         </is>
       </c>
     </row>
@@ -922,7 +922,7 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>2026-10-01 10:50:17</t>
+          <t>2026-10-08 16:16:03</t>
         </is>
       </c>
     </row>
@@ -940,7 +940,7 @@
       <c r="C27" t="inlineStr"/>
       <c r="D27" t="inlineStr">
         <is>
-          <t>2026-10-01 10:50:17</t>
+          <t>2026-10-08 16:16:03</t>
         </is>
       </c>
     </row>
@@ -958,7 +958,7 @@
       <c r="C28" t="inlineStr"/>
       <c r="D28" t="inlineStr">
         <is>
-          <t>2026-10-01 10:50:17</t>
+          <t>2026-10-08 16:16:03</t>
         </is>
       </c>
     </row>
@@ -976,7 +976,7 @@
       <c r="C29" t="inlineStr"/>
       <c r="D29" t="inlineStr">
         <is>
-          <t>2026-10-01 10:50:17</t>
+          <t>2026-10-08 16:16:03</t>
         </is>
       </c>
     </row>
@@ -994,7 +994,7 @@
       <c r="C30" t="inlineStr"/>
       <c r="D30" t="inlineStr">
         <is>
-          <t>2026-10-01 10:50:17</t>
+          <t>2026-10-08 16:16:03</t>
         </is>
       </c>
     </row>
@@ -1012,7 +1012,7 @@
       <c r="C31" t="inlineStr"/>
       <c r="D31" t="inlineStr">
         <is>
-          <t>2026-10-01 10:50:17</t>
+          <t>2026-10-08 16:16:03</t>
         </is>
       </c>
     </row>
@@ -1034,7 +1034,7 @@
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>2026-10-01 10:50:17</t>
+          <t>2026-10-08 16:16:03</t>
         </is>
       </c>
     </row>
@@ -1052,7 +1052,7 @@
       <c r="C33" t="inlineStr"/>
       <c r="D33" t="inlineStr">
         <is>
-          <t>2026-10-01 10:50:17</t>
+          <t>2026-10-08 16:16:03</t>
         </is>
       </c>
     </row>
@@ -1070,7 +1070,7 @@
       <c r="C34" t="inlineStr"/>
       <c r="D34" t="inlineStr">
         <is>
-          <t>2026-10-01 10:50:17</t>
+          <t>2026-10-08 16:16:03</t>
         </is>
       </c>
     </row>
@@ -1088,7 +1088,7 @@
       <c r="C35" t="inlineStr"/>
       <c r="D35" t="inlineStr">
         <is>
-          <t>2026-10-01 10:50:17</t>
+          <t>2026-10-08 16:16:03</t>
         </is>
       </c>
     </row>
@@ -1110,7 +1110,7 @@
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>2026-10-01 10:50:17</t>
+          <t>2026-10-08 16:16:03</t>
         </is>
       </c>
     </row>
@@ -1128,7 +1128,7 @@
       <c r="C37" t="inlineStr"/>
       <c r="D37" t="inlineStr">
         <is>
-          <t>2026-10-01 10:50:17</t>
+          <t>2026-10-08 16:16:03</t>
         </is>
       </c>
     </row>
@@ -1146,7 +1146,7 @@
       <c r="C38" t="inlineStr"/>
       <c r="D38" t="inlineStr">
         <is>
-          <t>2026-10-01 10:50:17</t>
+          <t>2026-10-08 16:16:03</t>
         </is>
       </c>
     </row>
@@ -1164,7 +1164,7 @@
       <c r="C39" t="inlineStr"/>
       <c r="D39" t="inlineStr">
         <is>
-          <t>2026-10-01 10:50:17</t>
+          <t>2026-10-08 16:16:03</t>
         </is>
       </c>
     </row>
@@ -1182,7 +1182,7 @@
       <c r="C40" t="inlineStr"/>
       <c r="D40" t="inlineStr">
         <is>
-          <t>2026-10-01 10:50:17</t>
+          <t>2026-10-08 16:16:03</t>
         </is>
       </c>
     </row>
@@ -1200,7 +1200,7 @@
       <c r="C41" t="inlineStr"/>
       <c r="D41" t="inlineStr">
         <is>
-          <t>2026-10-01 10:50:17</t>
+          <t>2026-10-08 16:16:03</t>
         </is>
       </c>
     </row>
@@ -1218,7 +1218,7 @@
       <c r="C42" t="inlineStr"/>
       <c r="D42" t="inlineStr">
         <is>
-          <t>2026-10-01 10:50:17</t>
+          <t>2026-10-08 16:16:03</t>
         </is>
       </c>
     </row>
@@ -1236,7 +1236,7 @@
       <c r="C43" t="inlineStr"/>
       <c r="D43" t="inlineStr">
         <is>
-          <t>2026-10-01 10:50:17</t>
+          <t>2026-10-08 16:16:03</t>
         </is>
       </c>
     </row>
@@ -1254,7 +1254,7 @@
       <c r="C44" t="inlineStr"/>
       <c r="D44" t="inlineStr">
         <is>
-          <t>2026-10-01 10:50:17</t>
+          <t>2026-10-08 16:16:03</t>
         </is>
       </c>
     </row>
@@ -1276,7 +1276,7 @@
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>2026-10-01 10:50:17</t>
+          <t>2026-10-08 16:16:03</t>
         </is>
       </c>
     </row>
@@ -1298,7 +1298,7 @@
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>2026-10-01 10:50:17</t>
+          <t>2026-10-08 16:16:03</t>
         </is>
       </c>
     </row>
@@ -1316,7 +1316,7 @@
       <c r="C47" t="inlineStr"/>
       <c r="D47" t="inlineStr">
         <is>
-          <t>2026-10-01 10:50:17</t>
+          <t>2026-10-08 16:16:03</t>
         </is>
       </c>
     </row>
@@ -1334,7 +1334,7 @@
       <c r="C48" t="inlineStr"/>
       <c r="D48" t="inlineStr">
         <is>
-          <t>2026-10-01 10:50:17</t>
+          <t>2026-10-08 16:16:03</t>
         </is>
       </c>
     </row>
@@ -1352,7 +1352,7 @@
       <c r="C49" t="inlineStr"/>
       <c r="D49" t="inlineStr">
         <is>
-          <t>2026-10-01 10:50:17</t>
+          <t>2026-10-08 16:16:03</t>
         </is>
       </c>
     </row>
@@ -1370,7 +1370,7 @@
       <c r="C50" t="inlineStr"/>
       <c r="D50" t="inlineStr">
         <is>
-          <t>2026-10-01 10:50:17</t>
+          <t>2026-10-08 16:16:03</t>
         </is>
       </c>
     </row>
@@ -1388,7 +1388,7 @@
       <c r="C51" t="inlineStr"/>
       <c r="D51" t="inlineStr">
         <is>
-          <t>2026-10-01 10:50:17</t>
+          <t>2026-10-08 16:16:03</t>
         </is>
       </c>
     </row>
@@ -1406,7 +1406,7 @@
       <c r="C52" t="inlineStr"/>
       <c r="D52" t="inlineStr">
         <is>
-          <t>2026-10-01 10:50:17</t>
+          <t>2026-10-08 16:16:03</t>
         </is>
       </c>
     </row>
@@ -1424,7 +1424,7 @@
       <c r="C53" t="inlineStr"/>
       <c r="D53" t="inlineStr">
         <is>
-          <t>2026-10-01 10:50:17</t>
+          <t>2026-10-08 16:16:03</t>
         </is>
       </c>
     </row>
@@ -1442,7 +1442,7 @@
       <c r="C54" t="inlineStr"/>
       <c r="D54" t="inlineStr">
         <is>
-          <t>2026-10-01 10:50:17</t>
+          <t>2026-10-08 16:16:03</t>
         </is>
       </c>
     </row>
@@ -1460,7 +1460,7 @@
       <c r="C55" t="inlineStr"/>
       <c r="D55" t="inlineStr">
         <is>
-          <t>2026-10-01 10:50:17</t>
+          <t>2026-10-08 16:16:03</t>
         </is>
       </c>
     </row>
@@ -1478,7 +1478,7 @@
       <c r="C56" t="inlineStr"/>
       <c r="D56" t="inlineStr">
         <is>
-          <t>2026-10-01 10:50:17</t>
+          <t>2026-10-08 16:16:03</t>
         </is>
       </c>
     </row>
@@ -1496,7 +1496,7 @@
       <c r="C57" t="inlineStr"/>
       <c r="D57" t="inlineStr">
         <is>
-          <t>2026-10-01 10:50:17</t>
+          <t>2026-10-08 16:16:03</t>
         </is>
       </c>
     </row>
@@ -1514,7 +1514,7 @@
       <c r="C58" t="inlineStr"/>
       <c r="D58" t="inlineStr">
         <is>
-          <t>2026-10-01 10:50:17</t>
+          <t>2026-10-08 16:16:03</t>
         </is>
       </c>
     </row>
@@ -1532,7 +1532,7 @@
       <c r="C59" t="inlineStr"/>
       <c r="D59" t="inlineStr">
         <is>
-          <t>2026-10-01 10:50:17</t>
+          <t>2026-10-08 16:16:03</t>
         </is>
       </c>
     </row>
@@ -1554,7 +1554,7 @@
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>2026-10-01 10:50:17</t>
+          <t>2026-10-08 16:16:03</t>
         </is>
       </c>
     </row>
@@ -1576,7 +1576,7 @@
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>2026-10-01 10:50:17</t>
+          <t>2026-10-08 16:16:03</t>
         </is>
       </c>
     </row>
@@ -1598,7 +1598,7 @@
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>2026-10-01 10:50:17</t>
+          <t>2026-10-08 16:16:03</t>
         </is>
       </c>
     </row>
@@ -1616,7 +1616,7 @@
       <c r="C63" t="inlineStr"/>
       <c r="D63" t="inlineStr">
         <is>
-          <t>2026-10-01 10:50:17</t>
+          <t>2026-10-08 16:16:03</t>
         </is>
       </c>
     </row>
@@ -1634,7 +1634,7 @@
       <c r="C64" t="inlineStr"/>
       <c r="D64" t="inlineStr">
         <is>
-          <t>2026-10-01 10:50:17</t>
+          <t>2026-10-08 16:16:03</t>
         </is>
       </c>
     </row>
@@ -1652,7 +1652,7 @@
       <c r="C65" t="inlineStr"/>
       <c r="D65" t="inlineStr">
         <is>
-          <t>2026-10-01 10:50:17</t>
+          <t>2026-10-08 16:16:03</t>
         </is>
       </c>
     </row>
@@ -1670,7 +1670,7 @@
       <c r="C66" t="inlineStr"/>
       <c r="D66" t="inlineStr">
         <is>
-          <t>2026-10-01 10:50:17</t>
+          <t>2026-10-08 16:16:03</t>
         </is>
       </c>
     </row>
@@ -1688,7 +1688,7 @@
       <c r="C67" t="inlineStr"/>
       <c r="D67" t="inlineStr">
         <is>
-          <t>2026-10-01 10:50:17</t>
+          <t>2026-10-08 16:16:03</t>
         </is>
       </c>
     </row>
@@ -1706,7 +1706,7 @@
       <c r="C68" t="inlineStr"/>
       <c r="D68" t="inlineStr">
         <is>
-          <t>2026-10-01 10:50:17</t>
+          <t>2026-10-08 16:16:03</t>
         </is>
       </c>
     </row>
@@ -1724,7 +1724,7 @@
       <c r="C69" t="inlineStr"/>
       <c r="D69" t="inlineStr">
         <is>
-          <t>2026-10-01 10:50:17</t>
+          <t>2026-10-08 16:16:03</t>
         </is>
       </c>
     </row>
@@ -1742,7 +1742,7 @@
       <c r="C70" t="inlineStr"/>
       <c r="D70" t="inlineStr">
         <is>
-          <t>2026-10-01 10:50:17</t>
+          <t>2026-10-08 16:16:03</t>
         </is>
       </c>
     </row>
@@ -1760,7 +1760,7 @@
       <c r="C71" t="inlineStr"/>
       <c r="D71" t="inlineStr">
         <is>
-          <t>2026-10-01 10:50:17</t>
+          <t>2026-10-08 16:16:03</t>
         </is>
       </c>
     </row>
@@ -1778,7 +1778,7 @@
       <c r="C72" t="inlineStr"/>
       <c r="D72" t="inlineStr">
         <is>
-          <t>2026-10-01 10:50:17</t>
+          <t>2026-10-08 16:16:03</t>
         </is>
       </c>
     </row>
@@ -1800,7 +1800,7 @@
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>2026-10-01 10:50:17</t>
+          <t>2026-10-08 16:16:03</t>
         </is>
       </c>
     </row>
@@ -1822,7 +1822,7 @@
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>2026-10-01 10:50:17</t>
+          <t>2026-10-08 16:16:03</t>
         </is>
       </c>
     </row>
@@ -1840,7 +1840,7 @@
       <c r="C75" t="inlineStr"/>
       <c r="D75" t="inlineStr">
         <is>
-          <t>2026-10-01 10:50:17</t>
+          <t>2026-10-08 16:16:03</t>
         </is>
       </c>
     </row>
@@ -1862,7 +1862,7 @@
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>2026-10-01 10:50:17</t>
+          <t>2026-10-08 16:16:03</t>
         </is>
       </c>
     </row>
@@ -1884,7 +1884,7 @@
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>2026-10-01 10:50:17</t>
+          <t>2026-10-08 16:16:03</t>
         </is>
       </c>
     </row>
@@ -1902,7 +1902,7 @@
       <c r="C78" t="inlineStr"/>
       <c r="D78" t="inlineStr">
         <is>
-          <t>2026-10-01 10:50:17</t>
+          <t>2026-10-08 16:16:03</t>
         </is>
       </c>
     </row>
@@ -1920,7 +1920,7 @@
       <c r="C79" t="inlineStr"/>
       <c r="D79" t="inlineStr">
         <is>
-          <t>2026-10-01 10:50:17</t>
+          <t>2026-10-08 16:16:03</t>
         </is>
       </c>
     </row>
@@ -1942,7 +1942,7 @@
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>2026-10-01 10:50:17</t>
+          <t>2026-10-08 16:16:03</t>
         </is>
       </c>
     </row>
@@ -1960,7 +1960,7 @@
       <c r="C81" t="inlineStr"/>
       <c r="D81" t="inlineStr">
         <is>
-          <t>2026-10-01 10:50:17</t>
+          <t>2026-10-08 16:16:03</t>
         </is>
       </c>
     </row>
@@ -1978,7 +1978,7 @@
       <c r="C82" t="inlineStr"/>
       <c r="D82" t="inlineStr">
         <is>
-          <t>2026-10-01 10:50:17</t>
+          <t>2026-10-08 16:16:03</t>
         </is>
       </c>
     </row>
@@ -2000,7 +2000,7 @@
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>2026-10-01 10:50:17</t>
+          <t>2026-10-08 16:16:03</t>
         </is>
       </c>
     </row>
@@ -2018,7 +2018,7 @@
       <c r="C84" t="inlineStr"/>
       <c r="D84" t="inlineStr">
         <is>
-          <t>2026-10-01 10:50:17</t>
+          <t>2026-10-08 16:16:03</t>
         </is>
       </c>
     </row>
@@ -2036,7 +2036,7 @@
       <c r="C85" t="inlineStr"/>
       <c r="D85" t="inlineStr">
         <is>
-          <t>2026-10-01 10:50:17</t>
+          <t>2026-10-08 16:16:03</t>
         </is>
       </c>
     </row>
@@ -2054,7 +2054,7 @@
       <c r="C86" t="inlineStr"/>
       <c r="D86" t="inlineStr">
         <is>
-          <t>2026-10-01 10:50:17</t>
+          <t>2026-10-08 16:16:03</t>
         </is>
       </c>
     </row>
@@ -2076,7 +2076,7 @@
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>2026-10-01 10:50:17</t>
+          <t>2026-10-08 16:16:03</t>
         </is>
       </c>
     </row>
@@ -2094,7 +2094,7 @@
       <c r="C88" t="inlineStr"/>
       <c r="D88" t="inlineStr">
         <is>
-          <t>2026-10-01 10:50:17</t>
+          <t>2026-10-08 16:16:03</t>
         </is>
       </c>
     </row>
@@ -2112,7 +2112,7 @@
       <c r="C89" t="inlineStr"/>
       <c r="D89" t="inlineStr">
         <is>
-          <t>2026-10-01 10:50:17</t>
+          <t>2026-10-08 16:16:03</t>
         </is>
       </c>
     </row>
@@ -2130,7 +2130,7 @@
       <c r="C90" t="inlineStr"/>
       <c r="D90" t="inlineStr">
         <is>
-          <t>2026-10-01 10:50:17</t>
+          <t>2026-10-08 16:16:03</t>
         </is>
       </c>
     </row>
@@ -2152,7 +2152,7 @@
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t>2026-10-01 10:50:17</t>
+          <t>2026-10-08 16:16:03</t>
         </is>
       </c>
     </row>
@@ -2170,7 +2170,7 @@
       <c r="C92" t="inlineStr"/>
       <c r="D92" t="inlineStr">
         <is>
-          <t>2026-10-01 10:50:17</t>
+          <t>2026-10-08 16:16:03</t>
         </is>
       </c>
     </row>
@@ -2188,7 +2188,7 @@
       <c r="C93" t="inlineStr"/>
       <c r="D93" t="inlineStr">
         <is>
-          <t>2026-10-01 10:50:17</t>
+          <t>2026-10-08 16:16:03</t>
         </is>
       </c>
     </row>
@@ -2206,7 +2206,7 @@
       <c r="C94" t="inlineStr"/>
       <c r="D94" t="inlineStr">
         <is>
-          <t>2026-10-01 10:50:17</t>
+          <t>2026-10-08 16:16:03</t>
         </is>
       </c>
     </row>
@@ -2224,7 +2224,7 @@
       <c r="C95" t="inlineStr"/>
       <c r="D95" t="inlineStr">
         <is>
-          <t>2026-10-01 10:50:17</t>
+          <t>2026-10-08 16:16:03</t>
         </is>
       </c>
     </row>
@@ -2242,7 +2242,7 @@
       <c r="C96" t="inlineStr"/>
       <c r="D96" t="inlineStr">
         <is>
-          <t>2026-10-01 10:50:17</t>
+          <t>2026-10-08 16:16:03</t>
         </is>
       </c>
     </row>
@@ -2260,7 +2260,7 @@
       <c r="C97" t="inlineStr"/>
       <c r="D97" t="inlineStr">
         <is>
-          <t>2026-10-01 10:50:17</t>
+          <t>2026-10-08 16:16:03</t>
         </is>
       </c>
     </row>
@@ -2278,7 +2278,7 @@
       <c r="C98" t="inlineStr"/>
       <c r="D98" t="inlineStr">
         <is>
-          <t>2026-10-01 10:50:17</t>
+          <t>2026-10-08 16:16:03</t>
         </is>
       </c>
     </row>
@@ -2296,7 +2296,7 @@
       <c r="C99" t="inlineStr"/>
       <c r="D99" t="inlineStr">
         <is>
-          <t>2026-10-01 10:50:17</t>
+          <t>2026-10-08 16:16:03</t>
         </is>
       </c>
     </row>
@@ -2318,7 +2318,7 @@
       </c>
       <c r="D100" t="inlineStr">
         <is>
-          <t>2026-10-01 10:50:17</t>
+          <t>2026-10-08 16:16:03</t>
         </is>
       </c>
     </row>
@@ -2336,7 +2336,7 @@
       <c r="C101" t="inlineStr"/>
       <c r="D101" t="inlineStr">
         <is>
-          <t>2026-10-01 10:50:17</t>
+          <t>2026-10-08 16:16:03</t>
         </is>
       </c>
     </row>
@@ -2358,7 +2358,7 @@
       </c>
       <c r="D102" t="inlineStr">
         <is>
-          <t>2026-10-01 10:50:17</t>
+          <t>2026-10-08 16:16:03</t>
         </is>
       </c>
     </row>
@@ -2376,7 +2376,7 @@
       <c r="C103" t="inlineStr"/>
       <c r="D103" t="inlineStr">
         <is>
-          <t>2026-10-01 10:50:17</t>
+          <t>2026-10-08 16:16:03</t>
         </is>
       </c>
     </row>
@@ -2394,7 +2394,7 @@
       <c r="C104" t="inlineStr"/>
       <c r="D104" t="inlineStr">
         <is>
-          <t>2026-10-01 10:50:17</t>
+          <t>2026-10-08 16:16:03</t>
         </is>
       </c>
     </row>
@@ -2416,7 +2416,7 @@
       </c>
       <c r="D105" t="inlineStr">
         <is>
-          <t>2026-10-01 10:50:17</t>
+          <t>2026-10-08 16:16:03</t>
         </is>
       </c>
     </row>
@@ -2438,7 +2438,7 @@
       </c>
       <c r="D106" t="inlineStr">
         <is>
-          <t>2026-10-01 10:50:17</t>
+          <t>2026-10-08 16:16:03</t>
         </is>
       </c>
     </row>
@@ -2456,7 +2456,7 @@
       <c r="C107" t="inlineStr"/>
       <c r="D107" t="inlineStr">
         <is>
-          <t>2026-10-01 10:50:17</t>
+          <t>2026-10-08 16:16:03</t>
         </is>
       </c>
     </row>
@@ -2474,7 +2474,7 @@
       <c r="C108" t="inlineStr"/>
       <c r="D108" t="inlineStr">
         <is>
-          <t>2026-10-01 10:50:17</t>
+          <t>2026-10-08 16:16:03</t>
         </is>
       </c>
     </row>
@@ -2492,7 +2492,7 @@
       <c r="C109" t="inlineStr"/>
       <c r="D109" t="inlineStr">
         <is>
-          <t>2026-10-01 10:50:17</t>
+          <t>2026-10-08 16:16:03</t>
         </is>
       </c>
     </row>
@@ -2510,7 +2510,7 @@
       <c r="C110" t="inlineStr"/>
       <c r="D110" t="inlineStr">
         <is>
-          <t>2026-10-01 10:50:17</t>
+          <t>2026-10-08 16:16:03</t>
         </is>
       </c>
     </row>
@@ -2528,7 +2528,7 @@
       <c r="C111" t="inlineStr"/>
       <c r="D111" t="inlineStr">
         <is>
-          <t>2026-10-01 10:50:17</t>
+          <t>2026-10-08 16:16:03</t>
         </is>
       </c>
     </row>
@@ -2546,7 +2546,7 @@
       <c r="C112" t="inlineStr"/>
       <c r="D112" t="inlineStr">
         <is>
-          <t>2026-10-01 10:50:17</t>
+          <t>2026-10-08 16:16:03</t>
         </is>
       </c>
     </row>
@@ -2568,7 +2568,7 @@
       </c>
       <c r="D113" t="inlineStr">
         <is>
-          <t>2026-10-01 10:50:17</t>
+          <t>2026-10-08 16:16:03</t>
         </is>
       </c>
     </row>
@@ -2586,7 +2586,7 @@
       <c r="C114" t="inlineStr"/>
       <c r="D114" t="inlineStr">
         <is>
-          <t>2026-10-01 10:50:17</t>
+          <t>2026-10-08 16:16:03</t>
         </is>
       </c>
     </row>
@@ -2604,7 +2604,7 @@
       <c r="C115" t="inlineStr"/>
       <c r="D115" t="inlineStr">
         <is>
-          <t>2026-10-01 10:50:17</t>
+          <t>2026-10-08 16:16:03</t>
         </is>
       </c>
     </row>
@@ -2622,7 +2622,7 @@
       <c r="C116" t="inlineStr"/>
       <c r="D116" t="inlineStr">
         <is>
-          <t>2026-10-01 10:50:17</t>
+          <t>2026-10-08 16:16:03</t>
         </is>
       </c>
     </row>
@@ -2644,7 +2644,7 @@
       </c>
       <c r="D117" t="inlineStr">
         <is>
-          <t>2026-10-01 10:50:17</t>
+          <t>2026-10-08 16:16:03</t>
         </is>
       </c>
     </row>
@@ -2662,7 +2662,7 @@
       <c r="C118" t="inlineStr"/>
       <c r="D118" t="inlineStr">
         <is>
-          <t>2026-10-01 10:50:17</t>
+          <t>2026-10-08 16:16:03</t>
         </is>
       </c>
     </row>
@@ -2680,7 +2680,7 @@
       <c r="C119" t="inlineStr"/>
       <c r="D119" t="inlineStr">
         <is>
-          <t>2026-10-01 10:50:17</t>
+          <t>2026-10-08 16:16:03</t>
         </is>
       </c>
     </row>
@@ -2698,7 +2698,7 @@
       <c r="C120" t="inlineStr"/>
       <c r="D120" t="inlineStr">
         <is>
-          <t>2026-10-01 10:50:17</t>
+          <t>2026-10-08 16:16:03</t>
         </is>
       </c>
     </row>
@@ -2716,7 +2716,7 @@
       <c r="C121" t="inlineStr"/>
       <c r="D121" t="inlineStr">
         <is>
-          <t>2026-10-01 10:50:17</t>
+          <t>2026-10-08 16:16:03</t>
         </is>
       </c>
     </row>
@@ -2738,7 +2738,7 @@
       </c>
       <c r="D122" t="inlineStr">
         <is>
-          <t>2026-10-01 10:50:17</t>
+          <t>2026-10-08 16:16:03</t>
         </is>
       </c>
     </row>
@@ -2756,7 +2756,7 @@
       <c r="C123" t="inlineStr"/>
       <c r="D123" t="inlineStr">
         <is>
-          <t>2026-10-01 10:50:17</t>
+          <t>2026-10-08 16:16:03</t>
         </is>
       </c>
     </row>
@@ -2774,7 +2774,7 @@
       <c r="C124" t="inlineStr"/>
       <c r="D124" t="inlineStr">
         <is>
-          <t>2026-10-01 10:50:17</t>
+          <t>2026-10-08 16:16:03</t>
         </is>
       </c>
     </row>
@@ -2792,7 +2792,7 @@
       <c r="C125" t="inlineStr"/>
       <c r="D125" t="inlineStr">
         <is>
-          <t>2026-10-01 10:50:17</t>
+          <t>2026-10-08 16:16:03</t>
         </is>
       </c>
     </row>
@@ -2814,7 +2814,7 @@
       </c>
       <c r="D126" t="inlineStr">
         <is>
-          <t>2026-10-01 10:50:17</t>
+          <t>2026-10-08 16:16:03</t>
         </is>
       </c>
     </row>
@@ -2832,7 +2832,7 @@
       <c r="C127" t="inlineStr"/>
       <c r="D127" t="inlineStr">
         <is>
-          <t>2026-10-01 10:50:17</t>
+          <t>2026-10-08 16:16:03</t>
         </is>
       </c>
     </row>
@@ -2854,7 +2854,7 @@
       </c>
       <c r="D128" t="inlineStr">
         <is>
-          <t>2026-10-01 10:50:17</t>
+          <t>2026-10-08 16:16:03</t>
         </is>
       </c>
     </row>
@@ -2872,7 +2872,7 @@
       <c r="C129" t="inlineStr"/>
       <c r="D129" t="inlineStr">
         <is>
-          <t>2026-10-01 10:50:17</t>
+          <t>2026-10-08 16:16:03</t>
         </is>
       </c>
     </row>
@@ -2890,7 +2890,7 @@
       <c r="C130" t="inlineStr"/>
       <c r="D130" t="inlineStr">
         <is>
-          <t>2026-10-01 10:50:17</t>
+          <t>2026-10-08 16:16:03</t>
         </is>
       </c>
     </row>
@@ -2908,7 +2908,7 @@
       <c r="C131" t="inlineStr"/>
       <c r="D131" t="inlineStr">
         <is>
-          <t>2026-10-01 10:50:17</t>
+          <t>2026-10-08 16:16:03</t>
         </is>
       </c>
     </row>
@@ -2926,7 +2926,7 @@
       <c r="C132" t="inlineStr"/>
       <c r="D132" t="inlineStr">
         <is>
-          <t>2026-10-01 10:50:17</t>
+          <t>2026-10-08 16:16:03</t>
         </is>
       </c>
     </row>
@@ -2944,7 +2944,7 @@
       <c r="C133" t="inlineStr"/>
       <c r="D133" t="inlineStr">
         <is>
-          <t>2026-10-01 10:50:17</t>
+          <t>2026-10-08 16:16:03</t>
         </is>
       </c>
     </row>
@@ -2962,7 +2962,7 @@
       <c r="C134" t="inlineStr"/>
       <c r="D134" t="inlineStr">
         <is>
-          <t>2026-10-01 10:50:17</t>
+          <t>2026-10-08 16:16:03</t>
         </is>
       </c>
     </row>
@@ -2980,7 +2980,7 @@
       <c r="C135" t="inlineStr"/>
       <c r="D135" t="inlineStr">
         <is>
-          <t>2026-10-01 10:50:17</t>
+          <t>2026-10-08 16:16:03</t>
         </is>
       </c>
     </row>
@@ -2998,7 +2998,7 @@
       <c r="C136" t="inlineStr"/>
       <c r="D136" t="inlineStr">
         <is>
-          <t>2026-10-01 10:50:17</t>
+          <t>2026-10-08 16:16:03</t>
         </is>
       </c>
     </row>
@@ -3020,7 +3020,7 @@
       </c>
       <c r="D137" t="inlineStr">
         <is>
-          <t>2026-10-01 10:50:17</t>
+          <t>2026-10-08 16:16:03</t>
         </is>
       </c>
     </row>
@@ -3038,7 +3038,7 @@
       <c r="C138" t="inlineStr"/>
       <c r="D138" t="inlineStr">
         <is>
-          <t>2026-10-01 10:50:17</t>
+          <t>2026-10-08 16:16:03</t>
         </is>
       </c>
     </row>
@@ -3060,7 +3060,7 @@
       </c>
       <c r="D139" t="inlineStr">
         <is>
-          <t>2026-10-01 10:50:17</t>
+          <t>2026-10-08 16:16:03</t>
         </is>
       </c>
     </row>
@@ -3078,7 +3078,7 @@
       <c r="C140" t="inlineStr"/>
       <c r="D140" t="inlineStr">
         <is>
-          <t>2026-10-01 10:50:17</t>
+          <t>2026-10-08 16:16:03</t>
         </is>
       </c>
     </row>
@@ -3096,7 +3096,7 @@
       <c r="C141" t="inlineStr"/>
       <c r="D141" t="inlineStr">
         <is>
-          <t>2026-10-01 10:50:17</t>
+          <t>2026-10-08 16:16:03</t>
         </is>
       </c>
     </row>
@@ -3118,7 +3118,7 @@
       </c>
       <c r="D142" t="inlineStr">
         <is>
-          <t>2026-10-01 10:50:17</t>
+          <t>2026-10-08 16:16:03</t>
         </is>
       </c>
     </row>
@@ -3136,7 +3136,7 @@
       <c r="C143" t="inlineStr"/>
       <c r="D143" t="inlineStr">
         <is>
-          <t>2026-10-01 10:50:17</t>
+          <t>2026-10-08 16:16:03</t>
         </is>
       </c>
     </row>
@@ -3154,7 +3154,7 @@
       <c r="C144" t="inlineStr"/>
       <c r="D144" t="inlineStr">
         <is>
-          <t>2026-10-01 10:50:17</t>
+          <t>2026-10-08 16:16:03</t>
         </is>
       </c>
     </row>
@@ -3172,7 +3172,7 @@
       <c r="C145" t="inlineStr"/>
       <c r="D145" t="inlineStr">
         <is>
-          <t>2026-10-01 10:50:17</t>
+          <t>2026-10-08 16:16:03</t>
         </is>
       </c>
     </row>
@@ -3190,7 +3190,7 @@
       <c r="C146" t="inlineStr"/>
       <c r="D146" t="inlineStr">
         <is>
-          <t>2026-10-01 10:50:17</t>
+          <t>2026-10-08 16:16:03</t>
         </is>
       </c>
     </row>
@@ -3208,7 +3208,7 @@
       <c r="C147" t="inlineStr"/>
       <c r="D147" t="inlineStr">
         <is>
-          <t>2026-10-01 10:50:17</t>
+          <t>2026-10-08 16:16:03</t>
         </is>
       </c>
     </row>
@@ -3226,7 +3226,7 @@
       <c r="C148" t="inlineStr"/>
       <c r="D148" t="inlineStr">
         <is>
-          <t>2026-10-01 10:50:17</t>
+          <t>2026-10-08 16:16:03</t>
         </is>
       </c>
     </row>
@@ -3244,7 +3244,7 @@
       <c r="C149" t="inlineStr"/>
       <c r="D149" t="inlineStr">
         <is>
-          <t>2026-10-01 10:50:17</t>
+          <t>2026-10-08 16:16:03</t>
         </is>
       </c>
     </row>
@@ -3262,7 +3262,7 @@
       <c r="C150" t="inlineStr"/>
       <c r="D150" t="inlineStr">
         <is>
-          <t>2026-10-01 10:50:17</t>
+          <t>2026-10-08 16:16:03</t>
         </is>
       </c>
     </row>
@@ -3280,7 +3280,7 @@
       <c r="C151" t="inlineStr"/>
       <c r="D151" t="inlineStr">
         <is>
-          <t>2026-10-01 10:50:17</t>
+          <t>2026-10-08 16:16:03</t>
         </is>
       </c>
     </row>
@@ -3298,7 +3298,7 @@
       <c r="C152" t="inlineStr"/>
       <c r="D152" t="inlineStr">
         <is>
-          <t>2026-10-01 10:50:17</t>
+          <t>2026-10-08 16:16:03</t>
         </is>
       </c>
     </row>
@@ -3316,7 +3316,7 @@
       <c r="C153" t="inlineStr"/>
       <c r="D153" t="inlineStr">
         <is>
-          <t>2026-10-01 10:50:17</t>
+          <t>2026-10-08 16:16:03</t>
         </is>
       </c>
     </row>
@@ -3334,7 +3334,7 @@
       <c r="C154" t="inlineStr"/>
       <c r="D154" t="inlineStr">
         <is>
-          <t>2026-10-01 10:50:17</t>
+          <t>2026-10-08 16:16:03</t>
         </is>
       </c>
     </row>
@@ -3352,7 +3352,7 @@
       <c r="C155" t="inlineStr"/>
       <c r="D155" t="inlineStr">
         <is>
-          <t>2026-10-01 10:50:17</t>
+          <t>2026-10-08 16:16:03</t>
         </is>
       </c>
     </row>
@@ -3370,7 +3370,7 @@
       <c r="C156" t="inlineStr"/>
       <c r="D156" t="inlineStr">
         <is>
-          <t>2026-10-01 10:50:17</t>
+          <t>2026-10-08 16:16:03</t>
         </is>
       </c>
     </row>
@@ -3392,7 +3392,7 @@
       </c>
       <c r="D157" t="inlineStr">
         <is>
-          <t>2026-10-01 10:50:17</t>
+          <t>2026-10-08 16:16:03</t>
         </is>
       </c>
     </row>
@@ -3410,7 +3410,7 @@
       <c r="C158" t="inlineStr"/>
       <c r="D158" t="inlineStr">
         <is>
-          <t>2026-10-01 10:50:17</t>
+          <t>2026-10-08 16:16:03</t>
         </is>
       </c>
     </row>
@@ -3428,7 +3428,7 @@
       <c r="C159" t="inlineStr"/>
       <c r="D159" t="inlineStr">
         <is>
-          <t>2026-10-01 10:50:17</t>
+          <t>2026-10-08 16:16:03</t>
         </is>
       </c>
     </row>
@@ -3446,7 +3446,7 @@
       <c r="C160" t="inlineStr"/>
       <c r="D160" t="inlineStr">
         <is>
-          <t>2026-10-01 10:50:17</t>
+          <t>2026-10-08 16:16:03</t>
         </is>
       </c>
     </row>
@@ -3464,7 +3464,7 @@
       <c r="C161" t="inlineStr"/>
       <c r="D161" t="inlineStr">
         <is>
-          <t>2026-10-01 10:50:17</t>
+          <t>2026-10-08 16:16:03</t>
         </is>
       </c>
     </row>
@@ -3482,7 +3482,7 @@
       <c r="C162" t="inlineStr"/>
       <c r="D162" t="inlineStr">
         <is>
-          <t>2026-10-01 10:50:17</t>
+          <t>2026-10-08 16:16:03</t>
         </is>
       </c>
     </row>
@@ -3500,7 +3500,7 @@
       <c r="C163" t="inlineStr"/>
       <c r="D163" t="inlineStr">
         <is>
-          <t>2026-10-01 10:50:17</t>
+          <t>2026-10-08 16:16:03</t>
         </is>
       </c>
     </row>
@@ -3518,7 +3518,7 @@
       <c r="C164" t="inlineStr"/>
       <c r="D164" t="inlineStr">
         <is>
-          <t>2026-10-01 10:50:17</t>
+          <t>2026-10-08 16:16:03</t>
         </is>
       </c>
     </row>
@@ -3540,7 +3540,7 @@
       </c>
       <c r="D165" t="inlineStr">
         <is>
-          <t>2026-10-01 10:50:17</t>
+          <t>2026-10-08 16:16:03</t>
         </is>
       </c>
     </row>
@@ -3558,7 +3558,7 @@
       <c r="C166" t="inlineStr"/>
       <c r="D166" t="inlineStr">
         <is>
-          <t>2026-10-01 10:50:17</t>
+          <t>2026-10-08 16:16:03</t>
         </is>
       </c>
     </row>
@@ -3580,7 +3580,7 @@
       </c>
       <c r="D167" t="inlineStr">
         <is>
-          <t>2026-10-01 10:50:17</t>
+          <t>2026-10-08 16:16:03</t>
         </is>
       </c>
     </row>
@@ -3598,7 +3598,7 @@
       <c r="C168" t="inlineStr"/>
       <c r="D168" t="inlineStr">
         <is>
-          <t>2026-10-01 10:50:17</t>
+          <t>2026-10-08 16:16:03</t>
         </is>
       </c>
     </row>
@@ -3616,7 +3616,7 @@
       <c r="C169" t="inlineStr"/>
       <c r="D169" t="inlineStr">
         <is>
-          <t>2026-10-01 10:50:17</t>
+          <t>2026-10-08 16:16:03</t>
         </is>
       </c>
     </row>
@@ -3634,7 +3634,7 @@
       <c r="C170" t="inlineStr"/>
       <c r="D170" t="inlineStr">
         <is>
-          <t>2026-10-01 10:50:17</t>
+          <t>2026-10-08 16:16:03</t>
         </is>
       </c>
     </row>
@@ -3656,7 +3656,7 @@
       </c>
       <c r="D171" t="inlineStr">
         <is>
-          <t>2026-10-01 10:50:17</t>
+          <t>2026-10-08 16:16:03</t>
         </is>
       </c>
     </row>
@@ -3674,7 +3674,7 @@
       <c r="C172" t="inlineStr"/>
       <c r="D172" t="inlineStr">
         <is>
-          <t>2026-10-01 10:50:17</t>
+          <t>2026-10-08 16:16:03</t>
         </is>
       </c>
     </row>
@@ -3692,7 +3692,7 @@
       <c r="C173" t="inlineStr"/>
       <c r="D173" t="inlineStr">
         <is>
-          <t>2026-10-01 10:50:17</t>
+          <t>2026-10-08 16:16:03</t>
         </is>
       </c>
     </row>
@@ -3710,7 +3710,7 @@
       <c r="C174" t="inlineStr"/>
       <c r="D174" t="inlineStr">
         <is>
-          <t>2026-10-01 10:50:17</t>
+          <t>2026-10-08 16:16:03</t>
         </is>
       </c>
     </row>
@@ -3732,7 +3732,7 @@
       </c>
       <c r="D175" t="inlineStr">
         <is>
-          <t>2026-10-01 10:50:17</t>
+          <t>2026-10-08 16:16:03</t>
         </is>
       </c>
     </row>
@@ -3750,7 +3750,7 @@
       <c r="C176" t="inlineStr"/>
       <c r="D176" t="inlineStr">
         <is>
-          <t>2026-10-01 10:50:17</t>
+          <t>2026-10-08 16:16:03</t>
         </is>
       </c>
     </row>
@@ -3772,7 +3772,7 @@
       </c>
       <c r="D177" t="inlineStr">
         <is>
-          <t>2026-10-01 10:50:17</t>
+          <t>2026-10-08 16:16:03</t>
         </is>
       </c>
     </row>
@@ -3790,7 +3790,7 @@
       <c r="C178" t="inlineStr"/>
       <c r="D178" t="inlineStr">
         <is>
-          <t>2026-10-01 10:50:17</t>
+          <t>2026-10-08 16:16:03</t>
         </is>
       </c>
     </row>
@@ -3808,7 +3808,7 @@
       <c r="C179" t="inlineStr"/>
       <c r="D179" t="inlineStr">
         <is>
-          <t>2026-10-01 10:50:17</t>
+          <t>2026-10-08 16:16:03</t>
         </is>
       </c>
     </row>
@@ -3826,7 +3826,7 @@
       <c r="C180" t="inlineStr"/>
       <c r="D180" t="inlineStr">
         <is>
-          <t>2026-10-01 10:50:17</t>
+          <t>2026-10-08 16:16:03</t>
         </is>
       </c>
     </row>
@@ -3848,7 +3848,7 @@
       </c>
       <c r="D181" t="inlineStr">
         <is>
-          <t>2026-10-01 10:50:17</t>
+          <t>2026-10-08 16:16:03</t>
         </is>
       </c>
     </row>
@@ -3866,7 +3866,7 @@
       <c r="C182" t="inlineStr"/>
       <c r="D182" t="inlineStr">
         <is>
-          <t>2026-10-01 10:50:17</t>
+          <t>2026-10-08 16:16:03</t>
         </is>
       </c>
     </row>
@@ -3888,7 +3888,7 @@
       </c>
       <c r="D183" t="inlineStr">
         <is>
-          <t>2026-10-01 10:50:17</t>
+          <t>2026-10-08 16:16:03</t>
         </is>
       </c>
     </row>
@@ -3906,7 +3906,7 @@
       <c r="C184" t="inlineStr"/>
       <c r="D184" t="inlineStr">
         <is>
-          <t>2026-10-01 10:50:17</t>
+          <t>2026-10-08 16:16:03</t>
         </is>
       </c>
     </row>
@@ -3928,7 +3928,7 @@
       </c>
       <c r="D185" t="inlineStr">
         <is>
-          <t>2026-10-01 10:50:17</t>
+          <t>2026-10-08 16:16:03</t>
         </is>
       </c>
     </row>
@@ -3946,7 +3946,7 @@
       <c r="C186" t="inlineStr"/>
       <c r="D186" t="inlineStr">
         <is>
-          <t>2026-10-01 10:50:17</t>
+          <t>2026-10-08 16:16:03</t>
         </is>
       </c>
     </row>
@@ -3968,7 +3968,7 @@
       </c>
       <c r="D187" t="inlineStr">
         <is>
-          <t>2026-10-01 10:50:17</t>
+          <t>2026-10-08 16:16:03</t>
         </is>
       </c>
     </row>
@@ -3990,7 +3990,7 @@
       </c>
       <c r="D188" t="inlineStr">
         <is>
-          <t>2026-10-01 10:50:17</t>
+          <t>2026-10-08 16:16:03</t>
         </is>
       </c>
     </row>
@@ -4008,7 +4008,7 @@
       <c r="C189" t="inlineStr"/>
       <c r="D189" t="inlineStr">
         <is>
-          <t>2026-10-01 10:50:17</t>
+          <t>2026-10-08 16:16:03</t>
         </is>
       </c>
     </row>
@@ -4026,7 +4026,7 @@
       <c r="C190" t="inlineStr"/>
       <c r="D190" t="inlineStr">
         <is>
-          <t>2026-10-01 10:50:17</t>
+          <t>2026-10-08 16:16:03</t>
         </is>
       </c>
     </row>
@@ -4044,7 +4044,7 @@
       <c r="C191" t="inlineStr"/>
       <c r="D191" t="inlineStr">
         <is>
-          <t>2026-10-01 10:50:17</t>
+          <t>2026-10-08 16:16:03</t>
         </is>
       </c>
     </row>
@@ -4066,7 +4066,7 @@
       </c>
       <c r="D192" t="inlineStr">
         <is>
-          <t>2026-10-01 10:50:17</t>
+          <t>2026-10-08 16:16:03</t>
         </is>
       </c>
     </row>
@@ -4084,7 +4084,7 @@
       <c r="C193" t="inlineStr"/>
       <c r="D193" t="inlineStr">
         <is>
-          <t>2026-10-01 10:50:17</t>
+          <t>2026-10-08 16:16:03</t>
         </is>
       </c>
     </row>
@@ -4106,7 +4106,7 @@
       </c>
       <c r="D194" t="inlineStr">
         <is>
-          <t>2026-10-01 10:50:17</t>
+          <t>2026-10-08 16:16:03</t>
         </is>
       </c>
     </row>
@@ -4124,7 +4124,7 @@
       <c r="C195" t="inlineStr"/>
       <c r="D195" t="inlineStr">
         <is>
-          <t>2026-10-01 10:50:17</t>
+          <t>2026-10-08 16:16:03</t>
         </is>
       </c>
     </row>
@@ -4142,7 +4142,7 @@
       <c r="C196" t="inlineStr"/>
       <c r="D196" t="inlineStr">
         <is>
-          <t>2026-10-01 10:50:17</t>
+          <t>2026-10-08 16:16:03</t>
         </is>
       </c>
     </row>
@@ -4160,7 +4160,7 @@
       <c r="C197" t="inlineStr"/>
       <c r="D197" t="inlineStr">
         <is>
-          <t>2026-10-01 10:50:17</t>
+          <t>2026-10-08 16:16:03</t>
         </is>
       </c>
     </row>
@@ -4182,7 +4182,7 @@
       </c>
       <c r="D198" t="inlineStr">
         <is>
-          <t>2026-10-01 10:50:17</t>
+          <t>2026-10-08 16:16:03</t>
         </is>
       </c>
     </row>
@@ -4200,7 +4200,7 @@
       <c r="C199" t="inlineStr"/>
       <c r="D199" t="inlineStr">
         <is>
-          <t>2026-10-01 10:50:17</t>
+          <t>2026-10-08 16:16:03</t>
         </is>
       </c>
     </row>
@@ -4218,7 +4218,7 @@
       <c r="C200" t="inlineStr"/>
       <c r="D200" t="inlineStr">
         <is>
-          <t>2026-10-01 10:50:17</t>
+          <t>2026-10-08 16:16:03</t>
         </is>
       </c>
     </row>
@@ -4236,7 +4236,7 @@
       <c r="C201" t="inlineStr"/>
       <c r="D201" t="inlineStr">
         <is>
-          <t>2026-10-01 10:50:17</t>
+          <t>2026-10-08 16:16:03</t>
         </is>
       </c>
     </row>
@@ -4254,7 +4254,7 @@
       <c r="C202" t="inlineStr"/>
       <c r="D202" t="inlineStr">
         <is>
-          <t>2026-10-01 10:50:17</t>
+          <t>2026-10-08 16:16:03</t>
         </is>
       </c>
     </row>
@@ -4272,7 +4272,7 @@
       <c r="C203" t="inlineStr"/>
       <c r="D203" t="inlineStr">
         <is>
-          <t>2026-10-01 10:50:17</t>
+          <t>2026-10-08 16:16:03</t>
         </is>
       </c>
     </row>
@@ -4290,7 +4290,7 @@
       <c r="C204" t="inlineStr"/>
       <c r="D204" t="inlineStr">
         <is>
-          <t>2026-10-01 10:50:17</t>
+          <t>2026-10-08 16:16:03</t>
         </is>
       </c>
     </row>
@@ -4308,7 +4308,7 @@
       <c r="C205" t="inlineStr"/>
       <c r="D205" t="inlineStr">
         <is>
-          <t>2026-10-01 10:50:17</t>
+          <t>2026-10-08 16:16:03</t>
         </is>
       </c>
     </row>
@@ -4326,7 +4326,7 @@
       <c r="C206" t="inlineStr"/>
       <c r="D206" t="inlineStr">
         <is>
-          <t>2026-10-01 10:50:17</t>
+          <t>2026-10-08 16:16:03</t>
         </is>
       </c>
     </row>
@@ -4348,7 +4348,7 @@
       </c>
       <c r="D207" t="inlineStr">
         <is>
-          <t>2026-10-01 10:50:17</t>
+          <t>2026-10-08 16:16:03</t>
         </is>
       </c>
     </row>
@@ -4366,7 +4366,7 @@
       <c r="C208" t="inlineStr"/>
       <c r="D208" t="inlineStr">
         <is>
-          <t>2026-10-01 10:50:17</t>
+          <t>2026-10-08 16:16:03</t>
         </is>
       </c>
     </row>
@@ -4384,7 +4384,7 @@
       <c r="C209" t="inlineStr"/>
       <c r="D209" t="inlineStr">
         <is>
-          <t>2026-10-01 10:50:17</t>
+          <t>2026-10-08 16:16:03</t>
         </is>
       </c>
     </row>

</xml_diff>